<commit_message>
Update PesticideDB curation UI and data
</commit_message>
<xml_diff>
--- a/data_files/core/no_evidence_pesticide.xlsx
+++ b/data_files/core/no_evidence_pesticide.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A136"/>
+  <dimension ref="A1:A135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,943 +438,936 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1,4-Dimethylnaphthalene</t>
+          <t>Afidopyropen</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Afidopyropen</t>
+          <t>Aldicarb</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aldicarb</t>
+          <t>Aminocyclopyrachlor</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Aminocyclopyrachlor</t>
+          <t>Aminopyralid</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aminopyralid</t>
+          <t>Amitraz</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Amitraz</t>
+          <t>Amitrole</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Amitrole</t>
+          <t>Azocyclotin</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Azocyclotin</t>
+          <t>Benalaxyl</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Benalaxyl</t>
+          <t>Benzovindiflupyr</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Benzovindiflupyr</t>
+          <t>Benzpyrimoxan</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Benzpyrimoxan</t>
+          <t>Bicyclopyrone</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Bicyclopyrone</t>
+          <t>Bifenazate</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Bifenazate</t>
+          <t>Bitertanol</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bitertanol</t>
+          <t>Bixafen</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bixafen</t>
+          <t>Broflanilide</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Broflanilide</t>
+          <t>Chlorfenapyr</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Chlorfenapyr</t>
+          <t>Chlormequat</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Chlormequat</t>
+          <t>Clethodim</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Clethodim</t>
+          <t>Clofentezine</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Clofentezine</t>
+          <t>Cyantraniliprole</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cyantraniliprole</t>
+          <t>Cyazofamid</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cyazofamid</t>
+          <t>Cyclaniliprole</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cyclaniliprole</t>
+          <t>Cycloxydim</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cycloxydim</t>
+          <t>Cyflumetofen</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cyflumetofen</t>
+          <t>Cyhalothrin (includes lambda-cyhalothrin)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cyhalothrin (includes lambda-cyhalothrin)</t>
+          <t>Cyhexatin</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cyhexatin</t>
+          <t>Cyproconazole</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cyproconazole</t>
+          <t>Diflubenzuron</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Diflubenzuron</t>
+          <t>Dimethenamid-P</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dimethenamid-P</t>
+          <t>Dimethipin</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Dimethipin</t>
+          <t>Dinocap</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Dinocap</t>
+          <t>Disulfoton</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Disulfoton</t>
+          <t>Dithianon</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Dithianon</t>
+          <t>Dodine</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Dodine</t>
+          <t>Ethephon</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ethephon</t>
+          <t>Ethoxyquin</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ethoxyquin</t>
+          <t>Etofenprox</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Etofenprox</t>
+          <t>Famoxadone</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Famoxadone</t>
+          <t>Fenamidone</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Fenamidone</t>
+          <t>Fenazaquin</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Fenazaquin</t>
+          <t>Fenbuconazole</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Fenbuconazole</t>
+          <t>Fenbutatin Oxide</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Fenbutatin Oxide</t>
+          <t>Fenpicoxamid</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Fenpicoxamid</t>
+          <t>Fenpropimorph</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Fenpropimorph</t>
+          <t>Fenpyrazamine</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Fenpyrazamine</t>
+          <t>Fenpyroximate</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Fenpyroximate</t>
+          <t>Fenthion</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Fenthion</t>
+          <t>Florylpicoxamid</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Florylpicoxamid</t>
+          <t>Fluazaindolizine</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Fluazaindolizine</t>
+          <t>Fluazifop-p-butyl</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Fluazifop-p-butyl</t>
+          <t>Fluensulfone</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Fluensulfone</t>
+          <t>Flufenoxuron</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Flufenoxuron</t>
+          <t>Fluindapyr</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Fluindapyr</t>
+          <t>Flumethrin</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Flumethrin</t>
+          <t>Flumioxazin</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Flumioxazin</t>
+          <t>Fluopicolide</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Fluopicolide</t>
+          <t>Fluopyram</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Fluopyram</t>
+          <t>Flupyradifurone</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Flupyradifurone</t>
+          <t>Flusilazole</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Flusilazole</t>
+          <t>Flutianil</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Flutianil</t>
+          <t>Flutolanil</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Flutolanil</t>
+          <t>Flutriafol</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Flutriafol</t>
+          <t>Fosetyl Al</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Fosetyl Al</t>
+          <t>Hexythiazox</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Hexythiazox</t>
+          <t>Hydrogen Phosphide</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Hydrogen Phosphide</t>
+          <t>Imazalil</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Imazalil</t>
+          <t>Imazapic</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Imazapic</t>
+          <t>Imazapyr</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Imazapyr</t>
+          <t>Inpyrfluxam</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Inpyrfluxam</t>
+          <t>Isocycloseram</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Isocycloseram</t>
+          <t>Isofetamid</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Isofetamid</t>
+          <t>Isoflucypram</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Isoflucypram</t>
+          <t>Isoprothiolane</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Isoprothiolane</t>
+          <t>Isotianil</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Isotianil</t>
+          <t>Kresoxim-Methyl</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Kresoxim-Methyl</t>
+          <t>Lufenuron</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Lufenuron</t>
+          <t>Maleic Hydrazide</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Maleic Hydrazide</t>
+          <t>Mandestrobin</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Mandestrobin</t>
+          <t>Mefentrifluconazole</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Mefentrifluconazole</t>
+          <t>Mepiquat Chloride</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Mepiquat Chloride</t>
+          <t>Meptyldinocap</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Meptyldinocap</t>
+          <t>Metaflumizone</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Metaflumizone</t>
+          <t>Metalaxyl-M</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Metalaxyl-M</t>
+          <t>Metconazole</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Metconazole</t>
+          <t>Methiocarb</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Methiocarb</t>
+          <t>Methoxyfenozide</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Methoxyfenozide</t>
+          <t>Metrafenone</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Metrafenone</t>
+          <t>Myclobutanil</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Myclobutanil</t>
+          <t>Natamycin</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Natamycin</t>
+          <t>Norflurazon</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Norflurazon</t>
+          <t>Novaluron</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Novaluron</t>
+          <t>Omethoate</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Omethoate</t>
+          <t>Oxathiapiprolin</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Oxathiapiprolin</t>
+          <t>Oxydemeton-Methyl</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Oxydemeton-Methyl</t>
+          <t>Parathion</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Parathion</t>
+          <t>Penconazole</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Penconazole</t>
+          <t>Phenthoate</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Phenthoate</t>
+          <t>Phosalone</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Phosalone</t>
+          <t>Picoxystrobin</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Picoxystrobin</t>
+          <t>Piperonyl Butoxide</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Piperonyl Butoxide</t>
+          <t>Pirimicarb</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Pirimicarb</t>
+          <t>Pydiflumetofen</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Pydiflumetofen</t>
+          <t>Pyflubumide</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Pyflubumide</t>
+          <t>Pyrasulfotole</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Pyrasulfotole</t>
+          <t>Pyraziflumid</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Pyraziflumid</t>
+          <t>Pyrethrins</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Pyrethrins</t>
+          <t>Pyridate</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Pyridate</t>
+          <t>Pyrifluquinazon</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Pyrifluquinazon</t>
+          <t>Pyriofenone</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Pyriofenone</t>
+          <t>Pyriproxyfen</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Pyriproxyfen</t>
+          <t>Quinoxyfen</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Quinoxyfen</t>
+          <t>Saflufenacil</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Saflufenacil</t>
+          <t>Sedaxane</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Sedaxane</t>
+          <t>Spinosad</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Spinosad</t>
+          <t>Spiromesifen</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Spiromesifen</t>
+          <t>Spiropidion</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Spiropidion</t>
+          <t>Spirotetramat</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Spirotetramat</t>
+          <t>Sulfuryl fluoride</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Sulfuryl fluoride</t>
+          <t>Tebufenozide</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Tebufenozide</t>
+          <t>Terbufos</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Terbufos</t>
+          <t>Tetraniliprole</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Tetraniliprole</t>
+          <t>Tioxazafen</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Tioxazafen</t>
+          <t>Tolclofos-Methyl</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Tolclofos-Methyl</t>
+          <t>Tolfenpyrad</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Tolfenpyrad</t>
+          <t>Triadimefon</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Triadimefon</t>
+          <t>Triadimenol</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Triadimenol</t>
+          <t>Tricyclazole</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Tricyclazole</t>
+          <t>Triflumezopyrim</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Triflumezopyrim</t>
+          <t>Triflumizole</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Triflumizole</t>
+          <t>Triflumuron</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Triflumuron</t>
+          <t>Triforine</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Triforine</t>
+          <t>Trinexapac-ethyl</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Trinexapac-ethyl</t>
+          <t>Valifenalate</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
-        <is>
-          <t>Valifenalate</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
         <is>
           <t>Zoxamide</t>
         </is>

</xml_diff>